<commit_message>
fix(fuentes): plantillas de Miscellaneous con hoja "Fuentes" vacia (solo titulo y encabezado)
Las plantillas de inputs/Miscellaneous no tienen datos, asi que no pueden tener
fuentes: add_fuentes_sheet.py ahora les escribe la hoja con el titulo y el
encabezado pero sin filas (targets() marca las plantillas; run() les pasa []).
Los 8 A-O de los escenarios y A-Xtra_Storage siguen recibiendo la tabla completa.
Test: nueva verificacion de plantilla vacia. README de data_patches actualizado.
</commit_message>
<xml_diff>
--- a/inputs/Miscellaneous/A-O_Demand.xlsx
+++ b/inputs/Miscellaneous/A-O_Demand.xlsx
@@ -1016,7 +1016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="4" min="1" max="1"/>
@@ -1066,742 +1066,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="16" t="inlineStr">
-        <is>
-          <t>Demand_Projection</t>
-        </is>
-      </c>
-      <c r="B3" s="16" t="inlineStr">
-        <is>
-          <t>ELC{ISO}XX03 (demanda eléctrica de cada uno de los 19 países)</t>
-        </is>
-      </c>
-      <c r="C3" s="16" t="inlineStr">
-        <is>
-          <t>SpecifiedAnnualDemand</t>
-        </is>
-      </c>
-      <c r="D3" s="16" t="inlineStr">
-        <is>
-          <t>2023-2024</t>
-        </is>
-      </c>
-      <c r="E3" s="16" t="inlineStr">
-        <is>
-          <t>OLACDE – Generación eléctrica por fuente + OLACDE – Matriz de balance energético</t>
-        </is>
-      </c>
-      <c r="F3" s="16" t="inlineStr">
-        <is>
-          <t>Demanda base (PJ) = generación eléctrica total del país en 2023 y 2024 (estadística anual de OLACDE, GWh × 0.0036) + importaciones − exportaciones de electricidad del mismo año (matriz de balance energético de OLACDE). Barbados no tiene interconexión: intercambio cero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="16" t="inlineStr">
-        <is>
-          <t>Demand_Projection</t>
-        </is>
-      </c>
-      <c r="B4" s="16" t="inlineStr">
-        <is>
-          <t>ELC{ISO}XX03 (18 países; Haití se trata aparte)</t>
-        </is>
-      </c>
-      <c r="C4" s="16" t="inlineStr">
-        <is>
-          <t>SpecifiedAnnualDemand</t>
-        </is>
-      </c>
-      <c r="D4" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E4" s="16" t="inlineStr">
-        <is>
-          <t>Escenario de demanda alta de los documentos oficiales de planificación eléctrica de cada país (ver una fila por país)</t>
-        </is>
-      </c>
-      <c r="F4" s="16" t="inlineStr">
-        <is>
-          <t>Demanda(año) = demanda base OLACDE de 2024 × crecimiento acumulado, aplicando año a año la tasa de crecimiento del escenario de demanda alta de cada documento nacional. Bolivia, Ecuador, Nicaragua y Paraguay no publican un escenario alto: se usa su escenario central. Años fuera del horizonte del documento: se prolonga la tendencia con la tasa de crecimiento compuesta del tramo más cercano.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>Demand_Projection</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>ELCHTIXX03 (Haití)</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>SpecifiedAnnualDemand</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E5" s="16" t="inlineStr">
-        <is>
-          <t>IEA – World Energy Outlook 2025, escenario Net Zero Emissions (NZE) para los 19 países de la región</t>
-        </is>
-      </c>
-      <c r="F5" s="16" t="inlineStr">
-        <is>
-          <t>Haití no cuenta con un documento oficial de planificación en el conjunto de datos; se conserva la proyección de la IEA. Esto produce un salto de 3.35 a 6.67 PJ entre 2024 (dato OLACDE) y 2025 (dato IEA).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Argentina – ELCARGXX03 e interconexiones de Argentina</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E6" s="16" t="inlineStr">
-        <is>
-          <t>ARG_LyE_para_ET_2050.pdf – Lineamientos y Escenarios para la Transición Energética al 2050 (Secretaría de Energía de Argentina)</t>
-        </is>
-      </c>
-      <c r="F6" s="16" t="inlineStr">
-        <is>
-          <t>Escenario Ambicioso (E3), Tabla 2, p. 38; el escenario central es el Escenario Base (E1). Tramo 2022-2030 común a ambos, sección 7.2.1, pp. 29-30.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>Bolivia – ELCBOLXX03 e interconexiones de Bolivia</t>
-        </is>
-      </c>
-      <c r="C7" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E7" s="16" t="inlineStr">
-        <is>
-          <t>BOL_PER_2035.pdf – Plan Eléctrico Referencial 2035 (Bolivia)</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>Escenario Referencial, Tabla 8, pp. 34-36 y Anexo 4, p. 93. El documento no publica escenario alto: se usa el Referencial.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>Brasil – ELCBRAXX03 e interconexiones de Brasil</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E8" s="16" t="inlineStr">
-        <is>
-          <t>BRA_PDE2034_report.pdf – Plano Decenal de Expansão de Energia 2034 (EPE) y BRA_PNE2050.pdf – Plano Nacional de Energia 2050 (EPE)</t>
-        </is>
-      </c>
-      <c r="F8" s="16" t="inlineStr">
-        <is>
-          <t>Escenario alto: Cenário Superior del PDE 2034, Figura 2-23 / Box 2.2, p. 62 (4.0 % anual). Escenario central: Cenário de Referência, Tabela 2-3, p. 61, prolongado a 2050 con la Figura 9 del PNE 2050.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B9" s="16" t="inlineStr">
-        <is>
-          <t>Barbados – ELCBRBXX03</t>
-        </is>
-      </c>
-      <c r="C9" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E9" s="16" t="inlineStr">
-        <is>
-          <t>BAR_ActionPlan_Roadmap_2030.pdf – Barbados Action Plan / Roadmap 2030</t>
-        </is>
-      </c>
-      <c r="F9" s="16" t="inlineStr">
-        <is>
-          <t>Escenario High, sección 6.2, p. 35 (el documento es narrativo, sin tabla numérica). Escenario central: Base.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B10" s="16" t="inlineStr">
-        <is>
-          <t>Chile – ELCCHLXX03 e interconexiones de Chile</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D10" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E10" s="16" t="inlineStr">
-        <is>
-          <t>CHL_PELP_2023-2027.pdf – Planificación Energética de Largo Plazo 2023-2027 (Ministerio de Energía de Chile)</t>
-        </is>
-      </c>
-      <c r="F10" s="16" t="inlineStr">
-        <is>
-          <t>Escenario Transición Acelerada, Figura 28 (valores leídos del gráfico). Escenario central: Carbono Neutralidad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B11" s="16" t="inlineStr">
-        <is>
-          <t>Colombia – ELCCOLXX03 e interconexiones de Colombia</t>
-        </is>
-      </c>
-      <c r="C11" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D11" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E11" s="16" t="inlineStr">
-        <is>
-          <t>COL_Plan_Generacion_2025-2039.pdf – Plan de Expansión de Referencia Generación 2025-2039 (UPME)</t>
-        </is>
-      </c>
-      <c r="F11" s="16" t="inlineStr">
-        <is>
-          <t>Escenario IC Superior 68 %, Tablas 32 y 33, pp. 93 y 95. Escenario central: Demanda Media, Tablas 13, 30 y 31.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B12" s="16" t="inlineStr">
-        <is>
-          <t>Costa Rica – ELCCRIXX03 e interconexiones de Costa Rica</t>
-        </is>
-      </c>
-      <c r="C12" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D12" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E12" s="16" t="inlineStr">
-        <is>
-          <t>CRI_PEG_2024-2040.pdf – Plan de Expansión de la Generación 2024-2040 (ICE)</t>
-        </is>
-      </c>
-      <c r="F12" s="16" t="inlineStr">
-        <is>
-          <t>Escenario Alta – Generación SEN, Tabla 6.2, pp. 60-61. Escenario central: Media.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B13" s="16" t="inlineStr">
-        <is>
-          <t>República Dominicana – ELCDOMXX03 e interconexión con Haití</t>
-        </is>
-      </c>
-      <c r="C13" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D13" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E13" s="16" t="inlineStr">
-        <is>
-          <t>DOM_PEN_2022-2037.pdf – Plan Energético Nacional 2022-2037 (CNE)</t>
-        </is>
-      </c>
-      <c r="F13" s="16" t="inlineStr">
-        <is>
-          <t>Escenario Alternativo, capítulo 6.1.6, Tabla 182. Escenario central: Tendencial, Tabla 181.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B14" s="16" t="inlineStr">
-        <is>
-          <t>Ecuador – ELCECUXX03 e interconexiones de Ecuador</t>
-        </is>
-      </c>
-      <c r="C14" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D14" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E14" s="16" t="inlineStr">
-        <is>
-          <t>ECU_PME_2023-2032.pdf – Plan Maestro de Electricidad 2023-2032 (Ecuador)</t>
-        </is>
-      </c>
-      <c r="F14" s="16" t="inlineStr">
-        <is>
-          <t>Hipótesis 2 – Caso Base (demanda en bornes de generación), capítulo 3, Tabla 3-26, p. 106. El documento no publica escenario alto: se usa el Caso Base.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B15" s="16" t="inlineStr">
-        <is>
-          <t>Guatemala – ELCGTMXX03 e interconexiones de Guatemala</t>
-        </is>
-      </c>
-      <c r="C15" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D15" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E15" s="16" t="inlineStr">
-        <is>
-          <t>GTM_PEG_2020-2050.pdf – Plan de Expansión de la Generación 2020-2050 (MEM / CNEE)</t>
-        </is>
-      </c>
-      <c r="F15" s="16" t="inlineStr">
-        <is>
-          <t>Escenario ALTO, Tabla 1, p. 35 (serie anual 2020-2050 en GWh). Escenario central: MEDIO.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B16" s="16" t="inlineStr">
-        <is>
-          <t>Honduras – ELCHNDXX03 e interconexiones de Honduras</t>
-        </is>
-      </c>
-      <c r="C16" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D16" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E16" s="16" t="inlineStr">
-        <is>
-          <t>HND_PIEG_2026-2035.pdf – Plan Indicativo de Expansión de la Generación 2026-2035 (y su anexo Anexos_HND_PIEG_2026-2035.pdf)</t>
-        </is>
-      </c>
-      <c r="F16" s="16" t="inlineStr">
-        <is>
-          <t>Escenario Alta IC 95 %, Tabla 26, p. 54 y Anexo Tabla C-3, p. 38. Escenario central: Media, Tabla 25 y Tabla C-2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B17" s="16" t="inlineStr">
-        <is>
-          <t>Haití – ELCHTIXX03 (solo 2023-2024 con dato OLACDE)</t>
-        </is>
-      </c>
-      <c r="C17" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D17" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E17" s="16" t="inlineStr">
-        <is>
-          <t>Sin documento nacional; 2025-2050 según IEA World Energy Outlook 2025 (NZE)</t>
-        </is>
-      </c>
-      <c r="F17" s="16" t="inlineStr">
-        <is>
-          <t>Ver la fila de Haití en Demand_Projection.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B18" s="16" t="inlineStr">
-        <is>
-          <t>México – ELCMEXXX03 e interconexión con Guatemala</t>
-        </is>
-      </c>
-      <c r="C18" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D18" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E18" s="16" t="inlineStr">
-        <is>
-          <t>MEX_PRODESEN_2024-2038_cap1-6.pdf – Programa de Desarrollo del Sistema Eléctrico Nacional 2024-2038 (SENER)</t>
-        </is>
-      </c>
-      <c r="F18" s="16" t="inlineStr">
-        <is>
-          <t>Escenario Alto, Cuadro 3.4, p. 63 (tasa media anual 2.9 %). Escenario central: Planeación, Cuadros 3.1, 3.4 y 3.5, pp. 38, 63 y 64 (consumo neto del SEN).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B19" s="16" t="inlineStr">
-        <is>
-          <t>Nicaragua – ELCNICXX03 e interconexiones de Nicaragua</t>
-        </is>
-      </c>
-      <c r="C19" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D19" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E19" s="16" t="inlineStr">
-        <is>
-          <t>NIC_PIEG_2021-2035.pdf – Plan Indicativo de Expansión de la Generación 2021-2035 (MEM)</t>
-        </is>
-      </c>
-      <c r="F19" s="16" t="inlineStr">
-        <is>
-          <t>Demanda Media del SIN, Tabla 5, p. 10. El documento no publica escenario alto: se usa la Media.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B20" s="16" t="inlineStr">
-        <is>
-          <t>Panamá – ELCPANXX03 e interconexiones de Panamá</t>
-        </is>
-      </c>
-      <c r="C20" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D20" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E20" s="16" t="inlineStr">
-        <is>
-          <t>PAN_PESIN_2025-2039_TomoII.pdf – Plan de Expansión del Sistema Interconectado Nacional 2025-2039 Tomo II (ETESA)</t>
-        </is>
-      </c>
-      <c r="F20" s="16" t="inlineStr">
-        <is>
-          <t>Escenario Optimista-Alto, Tabla 2.1, p. 22. Escenario central: Moderado-Medio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B21" s="16" t="inlineStr">
-        <is>
-          <t>Perú – ELCPERXX03 e interconexiones de Perú</t>
-        </is>
-      </c>
-      <c r="C21" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D21" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E21" s="16" t="inlineStr">
-        <is>
-          <t>PER_Anexo-D1_ProyeccionesDemandaFuturosExtremos.pdf – Anexo D.1 del Informe COES/DP-02-2022 (Plan de Transmisión del SEIN 2023-2032)</t>
-        </is>
-      </c>
-      <c r="F21" s="16" t="inlineStr">
-        <is>
-          <t>Escenario Muy Optimista, Tabla D.12, p. 12. Escenario central: Base, Tabla D.8, p. 10. El documento llega a 2032; el resto se prolonga con la misma tasa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B22" s="16" t="inlineStr">
-        <is>
-          <t>Paraguay – ELCPRYXX03 e interconexiones de Paraguay</t>
-        </is>
-      </c>
-      <c r="C22" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D22" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E22" s="16" t="inlineStr">
-        <is>
-          <t>PRY_PlanMaestro_2024-2043.pdf – Plan Maestro de Generación 2024-2043 (ANDE)</t>
-        </is>
-      </c>
-      <c r="F22" s="16" t="inlineStr">
-        <is>
-          <t>Sección 4.1.2, Figura 4.7, curva DTM (valores leídos del gráfico; solo el año 2043 = 57 561 GWh está rotulado). El documento tiene una sola trayectoria de demanda: se usa como escenario alto y central.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B23" s="16" t="inlineStr">
-        <is>
-          <t>El Salvador – ELCSLVXX03 e interconexiones de El Salvador</t>
-        </is>
-      </c>
-      <c r="C23" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D23" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E23" s="16" t="inlineStr">
-        <is>
-          <t>SLV_PIEG_2024-2038.pdf – Plan Indicativo de la Expansión de la Generación 2024-2038 (CNE)</t>
-        </is>
-      </c>
-      <c r="F23" s="16" t="inlineStr">
-        <is>
-          <t>Demanda Alta, Tabla 14, pp. 46-47. Escenario central: Demanda Base, Tabla 8, pp. 34-35.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="16" t="inlineStr">
-        <is>
-          <t>Demanda por país (hoja Demand_Projection y escalamiento de interconexiones)</t>
-        </is>
-      </c>
-      <c r="B24" s="16" t="inlineStr">
-        <is>
-          <t>Uruguay – ELCURYXX03 e interconexiones de Uruguay</t>
-        </is>
-      </c>
-      <c r="C24" s="16" t="inlineStr">
-        <is>
-          <t>Crecimiento de la demanda – escenario alto</t>
-        </is>
-      </c>
-      <c r="D24" s="16" t="inlineStr">
-        <is>
-          <t>2025-2050</t>
-        </is>
-      </c>
-      <c r="E24" s="16" t="inlineStr">
-        <is>
-          <t>URY_PEG_2024-2043.pdf – Plan de Expansión de la Generación 2024-2043 (UTE)</t>
-        </is>
-      </c>
-      <c r="F24" s="16" t="inlineStr">
-        <is>
-          <t>Escenario PES nov/23 + Demanda 50 MW, Tabla I, sección 3.1, pp. 16-17. Escenario central: Incondicional + Demanda 50 MW.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="16" t="inlineStr">
-        <is>
-          <t>Profiles</t>
-        </is>
-      </c>
-      <c r="B25" s="16" t="inlineStr">
-        <is>
-          <t>ELC{ISO}{RR}01/02/03 (perfil horario de la demanda de cada país) × 12 bloques horarios</t>
-        </is>
-      </c>
-      <c r="C25" s="16" t="inlineStr">
-        <is>
-          <t>SpecifiedDemandProfile</t>
-        </is>
-      </c>
-      <c r="D25" s="16" t="inlineStr">
-        <is>
-          <t>2023-2050</t>
-        </is>
-      </c>
-      <c r="E25" s="16" t="inlineStr">
-        <is>
-          <t>OSeMOSYS Global (base de datos abierta del modelo eléctrico mundial OSeMOSYS Global)</t>
-        </is>
-      </c>
-      <c r="F25" s="16" t="inlineStr">
-        <is>
-          <t>Distribución de la demanda anual entre los 12 bloques horarios; normalizada para que la suma sea 1 en cada año.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>